<commit_message>
Update non-ideal problem data workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Datos Problemas no ideales.xlsx
+++ b/Datos Problemas no ideales.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TFG\ReactorApp toolbox\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TFM\Aplicación Matlab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B0EF74-8274-4674-8068-13F57507E4F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1595D60E-6ACE-49F5-892C-24F536A5CF55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -400,10 +400,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V24"/>
+  <dimension ref="A1:AB24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -449,7 +449,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <f t="shared" ref="A2:A14" si="0">_xlfn.XLOOKUP($D$3,$1:$1,3:3,"no",0,1)</f>
         <v>0</v>
@@ -500,8 +500,15 @@
       <c r="V2" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <f>AA2*EXP(-AA2/2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>0.4</v>
@@ -549,8 +556,16 @@
       <c r="V3">
         <v>15.37</v>
       </c>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA3">
+        <f>+AA2+1</f>
+        <v>1</v>
+      </c>
+      <c r="AB3">
+        <f t="shared" ref="AB3:AB22" si="2">AA3*EXP(-AA3/2)</f>
+        <v>0.60653065971263342</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>0.8</v>
@@ -596,8 +611,16 @@
       <c r="V4">
         <v>15.1</v>
       </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA4">
+        <f t="shared" ref="AA4:AA15" si="3">+AA3+1</f>
+        <v>2</v>
+      </c>
+      <c r="AB4">
+        <f t="shared" si="2"/>
+        <v>0.73575888234288467</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>1.2</v>
@@ -625,7 +648,7 @@
         <v>52</v>
       </c>
       <c r="O5">
-        <f t="shared" ref="O5:O21" si="2">+O4+1</f>
+        <f t="shared" ref="O5:O21" si="4">+O4+1</f>
         <v>2</v>
       </c>
       <c r="P5">
@@ -643,8 +666,16 @@
       <c r="V5">
         <v>12.15</v>
       </c>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA5">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="AB5">
+        <f t="shared" si="2"/>
+        <v>0.66939048044528948</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>1.6</v>
@@ -672,7 +703,7 @@
         <v>65</v>
       </c>
       <c r="O6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="P6">
@@ -690,8 +721,16 @@
       <c r="V6">
         <v>11.93</v>
       </c>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA6">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="AB6">
+        <f t="shared" si="2"/>
+        <v>0.54134113294645081</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -719,7 +758,7 @@
         <v>82</v>
       </c>
       <c r="O7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
       <c r="P7">
@@ -737,8 +776,16 @@
       <c r="V7">
         <v>9.6</v>
       </c>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA7">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="AB7">
+        <f t="shared" si="2"/>
+        <v>0.41042499311949399</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>2.4</v>
@@ -766,7 +813,7 @@
         <v>77</v>
       </c>
       <c r="O8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="P8">
@@ -784,8 +831,16 @@
       <c r="V8">
         <v>9.43</v>
       </c>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA8">
+        <f t="shared" si="3"/>
+        <v>6</v>
+      </c>
+      <c r="AB8">
+        <f t="shared" si="2"/>
+        <v>0.29872241020718365</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>2.8</v>
@@ -813,7 +868,7 @@
         <v>70</v>
       </c>
       <c r="O9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="P9">
@@ -831,8 +886,16 @@
       <c r="V9">
         <v>7.59</v>
       </c>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA9">
+        <f t="shared" si="3"/>
+        <v>7</v>
+      </c>
+      <c r="AB9">
+        <f t="shared" si="2"/>
+        <v>0.2113816839562295</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>3.2</v>
@@ -860,7 +923,7 @@
         <v>56</v>
       </c>
       <c r="O10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="P10">
@@ -878,8 +941,16 @@
       <c r="V10">
         <v>7.46</v>
       </c>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA10">
+        <f t="shared" si="3"/>
+        <v>8</v>
+      </c>
+      <c r="AB10">
+        <f t="shared" si="2"/>
+        <v>0.14652511110987343</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -907,7 +978,7 @@
         <v>47</v>
       </c>
       <c r="O11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
       <c r="P11">
@@ -925,8 +996,16 @@
       <c r="V11">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA11">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="AB11">
+        <f t="shared" si="2"/>
+        <v>9.9980968844180756E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>4.8</v>
@@ -954,7 +1033,7 @@
         <v>32</v>
       </c>
       <c r="O12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="P12">
@@ -972,8 +1051,16 @@
       <c r="V12">
         <v>5.24</v>
       </c>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA12">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="AB12">
+        <f t="shared" si="2"/>
+        <v>6.7379469990854673E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>5.6</v>
@@ -1001,7 +1088,7 @@
         <v>15</v>
       </c>
       <c r="O13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="P13">
@@ -1019,8 +1106,16 @@
       <c r="V13">
         <v>3.75</v>
       </c>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA13">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="AB13">
+        <f t="shared" si="2"/>
+        <v>4.4954485823104733E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>5.8</v>
@@ -1048,7 +1143,7 @@
         <v>7</v>
       </c>
       <c r="O14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>11</v>
       </c>
       <c r="P14">
@@ -1066,14 +1161,22 @@
       <c r="V14">
         <v>3.27</v>
       </c>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA14">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+      <c r="AB14">
+        <f t="shared" si="2"/>
+        <v>2.9745026119996302E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15">
-        <f t="shared" ref="A15:A23" si="3">IF(_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,1)=0,"",_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,1))</f>
+        <f t="shared" ref="A15:A23" si="5">IF(_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,1)=0,"",_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,1))</f>
         <v>8</v>
       </c>
       <c r="B15">
-        <f t="shared" ref="B15:B23" si="4">IF(_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,-1)=0,"",_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,-1))</f>
+        <f t="shared" ref="B15:B23" si="6">IF(_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,-1)=0,"",_xlfn.XLOOKUP($D$3,$1:$1,16:16,"no",0,-1))</f>
         <v>1.62</v>
       </c>
       <c r="F15">
@@ -1113,14 +1216,22 @@
       <c r="V15">
         <v>2.08</v>
       </c>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA15">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="AB15">
+        <f t="shared" si="2"/>
+        <v>1.954470950870844E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>9.1999999999999993</v>
       </c>
       <c r="B16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.03</v>
       </c>
       <c r="F16">
@@ -1130,7 +1241,7 @@
         <v>0.9</v>
       </c>
       <c r="O16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>13</v>
       </c>
       <c r="P16">
@@ -1148,18 +1259,26 @@
       <c r="V16">
         <v>1.62</v>
       </c>
-    </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA16">
+        <f t="shared" ref="AA16:AA22" si="7">+AA15+1</f>
+        <v>14</v>
+      </c>
+      <c r="AB16">
+        <f t="shared" si="2"/>
+        <v>1.2766347517763227E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>10.8</v>
       </c>
       <c r="B17">
+        <f t="shared" si="6"/>
+        <v>0.71</v>
+      </c>
+      <c r="O17">
         <f t="shared" si="4"/>
-        <v>0.71</v>
-      </c>
-      <c r="O17">
-        <f t="shared" si="2"/>
         <v>14</v>
       </c>
       <c r="P17">
@@ -1177,18 +1296,26 @@
       <c r="V17">
         <v>1.03</v>
       </c>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA17">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="AB17">
+        <f t="shared" si="2"/>
+        <v>8.2962655522175049E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>12.8</v>
       </c>
       <c r="B18">
+        <f t="shared" si="6"/>
+        <v>0.36</v>
+      </c>
+      <c r="O18">
         <f t="shared" si="4"/>
-        <v>0.36</v>
-      </c>
-      <c r="O18">
-        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="P18">
@@ -1206,18 +1333,26 @@
       <c r="V18">
         <v>0.71</v>
       </c>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA18">
+        <f t="shared" si="7"/>
+        <v>16</v>
+      </c>
+      <c r="AB18">
+        <f t="shared" si="2"/>
+        <v>5.3674020464401897E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>16.8</v>
       </c>
       <c r="B19">
+        <f t="shared" si="6"/>
+        <v>0.12</v>
+      </c>
+      <c r="O19">
         <f t="shared" si="4"/>
-        <v>0.12</v>
-      </c>
-      <c r="O19">
-        <f t="shared" si="2"/>
         <v>16</v>
       </c>
       <c r="P19">
@@ -1235,18 +1370,26 @@
       <c r="V19">
         <v>0.36</v>
       </c>
-    </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA19">
+        <f t="shared" si="7"/>
+        <v>17</v>
+      </c>
+      <c r="AB19">
+        <f t="shared" si="2"/>
+        <v>3.4589622731809508E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>20.8</v>
       </c>
       <c r="B20">
+        <f t="shared" si="6"/>
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="O20">
         <f t="shared" si="4"/>
-        <v>3.4000000000000002E-2</v>
-      </c>
-      <c r="O20">
-        <f t="shared" si="2"/>
         <v>17</v>
       </c>
       <c r="P20">
@@ -1264,18 +1407,26 @@
       <c r="V20">
         <v>0.12</v>
       </c>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA20">
+        <f t="shared" si="7"/>
+        <v>18</v>
+      </c>
+      <c r="AB20">
+        <f t="shared" si="2"/>
+        <v>2.221376473560232E-3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>24</v>
       </c>
       <c r="B21">
+        <f t="shared" si="6"/>
+        <v>1E-3</v>
+      </c>
+      <c r="O21">
         <f t="shared" si="4"/>
-        <v>1E-3</v>
-      </c>
-      <c r="O21">
-        <f t="shared" si="2"/>
         <v>18</v>
       </c>
       <c r="P21">
@@ -1293,14 +1444,22 @@
       <c r="V21">
         <v>3.4000000000000002E-2</v>
       </c>
-    </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA21">
+        <f t="shared" si="7"/>
+        <v>19</v>
+      </c>
+      <c r="AB21">
+        <f t="shared" si="2"/>
+        <v>1.4221847678663113E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B22" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R22">
@@ -1315,14 +1474,22 @@
       <c r="V22">
         <v>1E-3</v>
       </c>
-    </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="AA22">
+        <f t="shared" si="7"/>
+        <v>20</v>
+      </c>
+      <c r="AB22">
+        <f t="shared" si="2"/>
+        <v>9.0799859524969711E-4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B23" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R23">
@@ -1332,7 +1499,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="R24">
         <v>25</v>
       </c>

</xml_diff>